<commit_message>
changes for tenantid selector
</commit_message>
<xml_diff>
--- a/Data/FinalReport.xlsx
+++ b/Data/FinalReport.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<x:sst xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
+<x:sst xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
   <x:si>
     <x:t>WO creation</x:t>
   </x:si>
@@ -41,6 +41,9 @@
   </x:si>
   <x:si>
     <x:t>27-01-2021 12:14:18 PM</x:t>
+  </x:si>
+  <x:si>
+    <x:t>08-02-2021 02:38:37 PM</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -478,6 +481,20 @@
         <x:v>8</x:v>
       </x:c>
     </x:row>
+    <x:row r="7" spans="1:4">
+      <x:c r="A7" s="0" t="s">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="B7" s="0" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C7" s="0" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D7" s="0" t="s">
+        <x:v>9</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
   <x:pageMargins left="0.75" right="0.75" top="0.75" bottom="0.5" header="0.5" footer="0.75"/>

</xml_diff>